<commit_message>
alteração na configuração de tabelas e otimização dos arquivos xlsx para uso futuro em dashbords Power BI
</commit_message>
<xml_diff>
--- a/data/powerbi_export/cinema_financial_decade.xlsx
+++ b/data/powerbi_export/cinema_financial_decade.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,258 +464,572 @@
           <t>faturamento_ajustado</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>quantidade_blockbusters</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>maior_faturamento</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>maior_faturamento_ajustado</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>quantidade_filmes</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>roi_medio</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>roi_mediano</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>53761</v>
+        <v>194079</v>
       </c>
       <c r="B2" t="n">
-        <v>1910</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1284356</v>
-      </c>
-      <c r="D2" t="n">
-        <v>6784341.25</v>
-      </c>
-      <c r="E2" t="n">
-        <v>24.77488432871939</v>
-      </c>
-      <c r="F2" t="n">
-        <v>31819771.33689672</v>
-      </c>
-      <c r="G2" t="n">
-        <v>168081269.7153095</v>
-      </c>
+        <v>1870</v>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>85638</v>
+        <v>159897</v>
       </c>
       <c r="B3" t="n">
-        <v>1920</v>
-      </c>
-      <c r="C3" t="n">
-        <v>3390127.22</v>
-      </c>
-      <c r="D3" t="n">
-        <v>3046327.31</v>
-      </c>
-      <c r="E3" t="n">
-        <v>17.33886096358118</v>
-      </c>
-      <c r="F3" t="n">
-        <v>58780944.51643199</v>
-      </c>
-      <c r="G3" t="n">
-        <v>52819845.67765027</v>
-      </c>
+        <v>1880</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>408</v>
+        <v>49296</v>
       </c>
       <c r="B4" t="n">
-        <v>1930</v>
-      </c>
-      <c r="C4" t="n">
-        <v>974881</v>
-      </c>
-      <c r="D4" t="n">
-        <v>19558079.37</v>
-      </c>
-      <c r="E4" t="n">
-        <v>21.48181070442395</v>
-      </c>
-      <c r="F4" t="n">
-        <v>20942209.10133952</v>
-      </c>
-      <c r="G4" t="n">
-        <v>420142958.7684392</v>
-      </c>
+        <v>1890</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>73</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>10895</v>
+        <v>775</v>
       </c>
       <c r="B5" t="n">
-        <v>1940</v>
+        <v>1900</v>
       </c>
       <c r="C5" t="n">
-        <v>1636960.62</v>
-      </c>
-      <c r="D5" t="n">
-        <v>15411126.25</v>
-      </c>
-      <c r="E5" t="n">
-        <v>16.2377609023892</v>
-      </c>
-      <c r="F5" t="n">
-        <v>26580575.15418678</v>
-      </c>
-      <c r="G5" t="n">
-        <v>250242183.2840339</v>
-      </c>
+        <v>6742.5</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>79</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5801</v>
+        <v>53761</v>
       </c>
       <c r="B6" t="n">
-        <v>1950</v>
+        <v>1910</v>
       </c>
       <c r="C6" t="n">
-        <v>2395612.06</v>
+        <v>1284356</v>
       </c>
       <c r="D6" t="n">
-        <v>23579749.7</v>
+        <v>6784341.25</v>
       </c>
       <c r="E6" t="n">
-        <v>11.27480419364786</v>
+        <v>24.77488432871939</v>
       </c>
       <c r="F6" t="n">
-        <v>27010056.90044138</v>
+        <v>31819771.33689672</v>
       </c>
       <c r="G6" t="n">
-        <v>265857060.8027268</v>
+        <v>168081269.7153095</v>
+      </c>
+      <c r="H6" t="n">
+        <v>159</v>
+      </c>
+      <c r="I6" t="n">
+        <v>11000000</v>
+      </c>
+      <c r="J6" t="n">
+        <v>272523727.6159133</v>
+      </c>
+      <c r="K6" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" t="n">
+        <v>4648.38</v>
+      </c>
+      <c r="M6" t="n">
+        <v>3500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>649</v>
+        <v>85638</v>
       </c>
       <c r="B7" t="n">
-        <v>1960</v>
+        <v>1920</v>
       </c>
       <c r="C7" t="n">
-        <v>4827756.69</v>
+        <v>3390127.22</v>
       </c>
       <c r="D7" t="n">
-        <v>26623865.74</v>
+        <v>3046327.31</v>
       </c>
       <c r="E7" t="n">
-        <v>9.517463168306522</v>
+        <v>17.33886096358118</v>
       </c>
       <c r="F7" t="n">
-        <v>45947996.48262041</v>
+        <v>58780944.51643199</v>
       </c>
       <c r="G7" t="n">
-        <v>253391661.5783879</v>
+        <v>52819845.67765027</v>
+      </c>
+      <c r="H7" t="n">
+        <v>380</v>
+      </c>
+      <c r="I7" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="J7" t="n">
+        <v>381454941.198786</v>
+      </c>
+      <c r="K7" t="n">
+        <v>15</v>
+      </c>
+      <c r="L7" t="n">
+        <v>914.5</v>
+      </c>
+      <c r="M7" t="n">
+        <v>130.77</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>103</v>
+        <v>408</v>
       </c>
       <c r="B8" t="n">
-        <v>1970</v>
+        <v>1930</v>
       </c>
       <c r="C8" t="n">
-        <v>4363765.01</v>
+        <v>974881</v>
       </c>
       <c r="D8" t="n">
-        <v>47500679.07</v>
+        <v>19558079.37</v>
       </c>
       <c r="E8" t="n">
-        <v>5.815100671140939</v>
+        <v>21.48181070442395</v>
       </c>
       <c r="F8" t="n">
-        <v>25375732.83835235</v>
+        <v>20942209.10133952</v>
       </c>
       <c r="G8" t="n">
-        <v>276221230.7396074</v>
+        <v>420142958.7684392</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1143</v>
+      </c>
+      <c r="I8" t="n">
+        <v>400176459</v>
+      </c>
+      <c r="J8" t="n">
+        <v>8596514940.60467</v>
+      </c>
+      <c r="K8" t="n">
+        <v>34</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1103.98</v>
+      </c>
+      <c r="M8" t="n">
+        <v>280.76</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>78</v>
+        <v>10895</v>
       </c>
       <c r="B9" t="n">
-        <v>1980</v>
+        <v>1940</v>
       </c>
       <c r="C9" t="n">
-        <v>11368329.57</v>
+        <v>1636960.62</v>
       </c>
       <c r="D9" t="n">
-        <v>36517681.32</v>
+        <v>15411126.25</v>
       </c>
       <c r="E9" t="n">
-        <v>2.912065848472057</v>
+        <v>16.2377609023892</v>
       </c>
       <c r="F9" t="n">
-        <v>33105324.29497202</v>
+        <v>26580575.15418678</v>
       </c>
       <c r="G9" t="n">
-        <v>106341892.637358</v>
+        <v>250242183.2840339</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1362</v>
+      </c>
+      <c r="I9" t="n">
+        <v>267447150</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4342742875.725419</v>
+      </c>
+      <c r="K9" t="n">
+        <v>45</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1254.26</v>
+      </c>
+      <c r="M9" t="n">
+        <v>283.33</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>862</v>
+        <v>5801</v>
       </c>
       <c r="B10" t="n">
-        <v>1990</v>
+        <v>1950</v>
       </c>
       <c r="C10" t="n">
-        <v>26190648.41</v>
+        <v>2395612.06</v>
       </c>
       <c r="D10" t="n">
-        <v>64111293.13</v>
+        <v>23579749.7</v>
       </c>
       <c r="E10" t="n">
-        <v>2.032450445242409</v>
+        <v>11.27480419364786</v>
       </c>
       <c r="F10" t="n">
-        <v>53231195.0220919</v>
+        <v>27010056.90044138</v>
       </c>
       <c r="G10" t="n">
-        <v>130303026.2671351</v>
+        <v>265857060.8027268</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1902</v>
+      </c>
+      <c r="I10" t="n">
+        <v>572000000</v>
+      </c>
+      <c r="J10" t="n">
+        <v>6449187998.766574</v>
+      </c>
+      <c r="K10" t="n">
+        <v>74</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1063.86</v>
+      </c>
+      <c r="M10" t="n">
+        <v>357.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>19457</v>
+        <v>649</v>
       </c>
       <c r="B11" t="n">
-        <v>2000</v>
+        <v>1960</v>
       </c>
       <c r="C11" t="n">
-        <v>27203255.66</v>
+        <v>4827756.69</v>
       </c>
       <c r="D11" t="n">
-        <v>79558100.44</v>
+        <v>26623865.74</v>
       </c>
       <c r="E11" t="n">
-        <v>1.573832319893143</v>
+        <v>9.517463168306522</v>
       </c>
       <c r="F11" t="n">
-        <v>42813362.96402408</v>
+        <v>45947996.48262041</v>
       </c>
       <c r="G11" t="n">
-        <v>125211109.7817769</v>
+        <v>253391661.5783879</v>
+      </c>
+      <c r="H11" t="n">
+        <v>120</v>
+      </c>
+      <c r="I11" t="n">
+        <v>286214286</v>
+      </c>
+      <c r="J11" t="n">
+        <v>2724033925.248149</v>
+      </c>
+      <c r="K11" t="n">
+        <v>129</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1210.64</v>
+      </c>
+      <c r="M11" t="n">
+        <v>280</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
+        <v>103</v>
+      </c>
+      <c r="B12" t="n">
+        <v>1970</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4363765.01</v>
+      </c>
+      <c r="D12" t="n">
+        <v>47500679.07</v>
+      </c>
+      <c r="E12" t="n">
+        <v>5.815100671140939</v>
+      </c>
+      <c r="F12" t="n">
+        <v>25375732.83835235</v>
+      </c>
+      <c r="G12" t="n">
+        <v>276221230.7396074</v>
+      </c>
+      <c r="H12" t="n">
+        <v>154</v>
+      </c>
+      <c r="I12" t="n">
+        <v>775398007</v>
+      </c>
+      <c r="J12" t="n">
+        <v>4509017470.907047</v>
+      </c>
+      <c r="K12" t="n">
+        <v>185</v>
+      </c>
+      <c r="L12" t="n">
+        <v>3157.8</v>
+      </c>
+      <c r="M12" t="n">
+        <v>572.46</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>78</v>
+      </c>
+      <c r="B13" t="n">
+        <v>1980</v>
+      </c>
+      <c r="C13" t="n">
+        <v>11368329.57</v>
+      </c>
+      <c r="D13" t="n">
+        <v>36517681.32</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2.912065848472057</v>
+      </c>
+      <c r="F13" t="n">
+        <v>33105324.29497202</v>
+      </c>
+      <c r="G13" t="n">
+        <v>106341892.637358</v>
+      </c>
+      <c r="H13" t="n">
+        <v>182</v>
+      </c>
+      <c r="I13" t="n">
+        <v>792965326</v>
+      </c>
+      <c r="J13" t="n">
+        <v>2309167244.867111</v>
+      </c>
+      <c r="K13" t="n">
+        <v>517</v>
+      </c>
+      <c r="L13" t="n">
+        <v>434.05</v>
+      </c>
+      <c r="M13" t="n">
+        <v>144.93</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>862</v>
+      </c>
+      <c r="B14" t="n">
+        <v>1990</v>
+      </c>
+      <c r="C14" t="n">
+        <v>26190648.41</v>
+      </c>
+      <c r="D14" t="n">
+        <v>64111293.13</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2.032450445242409</v>
+      </c>
+      <c r="F14" t="n">
+        <v>53231195.0220919</v>
+      </c>
+      <c r="G14" t="n">
+        <v>130303026.2671351</v>
+      </c>
+      <c r="H14" t="n">
+        <v>257</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1845034188</v>
+      </c>
+      <c r="J14" t="n">
+        <v>3749940556.888067</v>
+      </c>
+      <c r="K14" t="n">
+        <v>920</v>
+      </c>
+      <c r="L14" t="n">
+        <v>690.27</v>
+      </c>
+      <c r="M14" t="n">
+        <v>75.64</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>19457</v>
+      </c>
+      <c r="B15" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C15" t="n">
+        <v>27203255.66</v>
+      </c>
+      <c r="D15" t="n">
+        <v>79558100.44</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.573832319893143</v>
+      </c>
+      <c r="F15" t="n">
+        <v>42813362.96402408</v>
+      </c>
+      <c r="G15" t="n">
+        <v>125211109.7817769</v>
+      </c>
+      <c r="H15" t="n">
+        <v>508</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2787965087</v>
+      </c>
+      <c r="J15" t="n">
+        <v>4387789560.654299</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1751</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1003.67</v>
+      </c>
+      <c r="M15" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
         <v>79782</v>
       </c>
-      <c r="B12" t="n">
+      <c r="B16" t="n">
         <v>2010</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C16" t="n">
         <v>25564266.61</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D16" t="n">
         <v>90898374.34999999</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E16" t="n">
         <v>1.28501556075329</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F16" t="n">
         <v>32850480.39309575</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G16" t="n">
         <v>116805825.4869277</v>
+      </c>
+      <c r="H16" t="n">
+        <v>582</v>
+      </c>
+      <c r="I16" t="n">
+        <v>2068223624</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2657699539.957561</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1610</v>
+      </c>
+      <c r="L16" t="n">
+        <v>448.22</v>
+      </c>
+      <c r="M16" t="n">
+        <v>110.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajuste na coluna de quantidade de blockbusters no notebook 18
</commit_message>
<xml_diff>
--- a/data/powerbi_export/cinema_financial_decade.xlsx
+++ b/data/powerbi_export/cinema_financial_decade.xlsx
@@ -507,9 +507,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="n">
-        <v>2</v>
-      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -528,9 +526,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
-        <v>4</v>
-      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -549,9 +545,7 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="n">
-        <v>73</v>
-      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -572,9 +566,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="n">
-        <v>79</v>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -604,7 +596,7 @@
         <v>168081269.7153095</v>
       </c>
       <c r="H6" t="n">
-        <v>159</v>
+        <v>1</v>
       </c>
       <c r="I6" t="n">
         <v>11000000</v>
@@ -645,7 +637,7 @@
         <v>52819845.67765027</v>
       </c>
       <c r="H7" t="n">
-        <v>380</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
         <v>22000000</v>
@@ -686,7 +678,7 @@
         <v>420142958.7684392</v>
       </c>
       <c r="H8" t="n">
-        <v>1143</v>
+        <v>2</v>
       </c>
       <c r="I8" t="n">
         <v>400176459</v>
@@ -727,7 +719,7 @@
         <v>250242183.2840339</v>
       </c>
       <c r="H9" t="n">
-        <v>1362</v>
+        <v>3</v>
       </c>
       <c r="I9" t="n">
         <v>267447150</v>
@@ -768,7 +760,7 @@
         <v>265857060.8027268</v>
       </c>
       <c r="H10" t="n">
-        <v>1902</v>
+        <v>4</v>
       </c>
       <c r="I10" t="n">
         <v>572000000</v>
@@ -809,7 +801,7 @@
         <v>253391661.5783879</v>
       </c>
       <c r="H11" t="n">
-        <v>120</v>
+        <v>7</v>
       </c>
       <c r="I11" t="n">
         <v>286214286</v>
@@ -850,7 +842,7 @@
         <v>276221230.7396074</v>
       </c>
       <c r="H12" t="n">
-        <v>154</v>
+        <v>10</v>
       </c>
       <c r="I12" t="n">
         <v>775398007</v>
@@ -891,7 +883,7 @@
         <v>106341892.637358</v>
       </c>
       <c r="H13" t="n">
-        <v>182</v>
+        <v>26</v>
       </c>
       <c r="I13" t="n">
         <v>792965326</v>
@@ -932,7 +924,7 @@
         <v>130303026.2671351</v>
       </c>
       <c r="H14" t="n">
-        <v>257</v>
+        <v>46</v>
       </c>
       <c r="I14" t="n">
         <v>1845034188</v>
@@ -973,7 +965,7 @@
         <v>125211109.7817769</v>
       </c>
       <c r="H15" t="n">
-        <v>508</v>
+        <v>88</v>
       </c>
       <c r="I15" t="n">
         <v>2787965087</v>
@@ -1014,7 +1006,7 @@
         <v>116805825.4869277</v>
       </c>
       <c r="H16" t="n">
-        <v>582</v>
+        <v>81</v>
       </c>
       <c r="I16" t="n">
         <v>2068223624</v>

</xml_diff>